<commit_message>
feat: Fase 8 hardening completo v1.0.0
- Seguridad: SecurityHeadersMiddleware (X-Content-Type-Options, X-Frame-Options,
  X-XSS-Protection, Referrer-Policy, Permissions-Policy)
- Seguridad: CORS restringido (sin wildcard), rate limiting slowapi en endpoints costosos
- Resiliencia: XMCircuitBreaker (CLOSED→OPEN→HALF_OPEN) con alertas Telegram
- Observabilidad: /health completo (DB, Redis, XM circuit, data freshness, predictions)
- Observabilidad: /health/live (liveness) y /health/ready (readiness) para K8s
- Dashboard: Error boundary 500/404 en Flask server
- Documentación: RUNBOOK_PRODUCCION.md completo (322 líneas)
- Tests: 150 passed, 0 failures, 3 skipped
- Performance: 20 simulaciones en 0.25s (13ms/sim)
- Regresión: 13 páginas dashboard HTTP 200, 9 endpoints API HTTP 200

Fases 0-8 completadas. Sistema en producción.
</commit_message>
<xml_diff>
--- a/data/onedrive/Comunidades_Energeticas_Avance.xlsx
+++ b/data/onedrive/Comunidades_Energeticas_Avance.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -3906,20 +3906,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8f154a8c-a0d7-469f-a565-81a8dee811c9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8f154a8c-a0d7-469f-a565-81a8dee811c9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4111,11 +4111,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0787518D-69BD-4E45-AC35-D1E5AC391598}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51E095F6-BF66-41A9-AB03-40D964033B2A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51E095F6-BF66-41A9-AB03-40D964033B2A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0787518D-69BD-4E45-AC35-D1E5AC391598}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
fix: CU usuario str+Br + SIMEM list->DataFrame + chatbot noticias + limpieza
- fix(costo_usuario_final): TypeError html.Br() concatenado a str en alerta metodologia
- fix(config_simem): obtener_listado_simem() retorna DataFrame con columnas CodigoVariable/Nombre
- feat(chatbot): widget flotante anclado bottom:20px, crece hacia arriba, posicion top:70%
- feat(home): carrusel noticias KPI esquina superior izquierda, auto-rotante cada 7s
- fix(alertas): eliminadas 2 alertas BALANCE_ENERGETICO falsas de BD
- chore: eliminar 3 archivos basura (colon, ettings, tructure.database.manager)
- chore(gitignore): ignorar archivos de pager/terminal accidentales
- docs(README): actualizar a v1.4.0, estado 15 Marzo 2026, 261 archivos Python
- refactor: mejoras en servicios de dominio, ETL, API y paginas de dashboard
</commit_message>
<xml_diff>
--- a/data/onedrive/Comunidades_Energeticas_Avance.xlsx
+++ b/data/onedrive/Comunidades_Energeticas_Avance.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29910"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -3906,20 +3906,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8f154a8c-a0d7-469f-a565-81a8dee811c9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8f154a8c-a0d7-469f-a565-81a8dee811c9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4111,11 +4111,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51E095F6-BF66-41A9-AB03-40D964033B2A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0787518D-69BD-4E45-AC35-D1E5AC391598}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0787518D-69BD-4E45-AC35-D1E5AC391598}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51E095F6-BF66-41A9-AB03-40D964033B2A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>